<commit_message>
Resolve "Milestone 2 enhancement/bug fixing"
</commit_message>
<xml_diff>
--- a/public/manifest/sample_manifest.xlsx
+++ b/public/manifest/sample_manifest.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
   <si>
     <t>name</t>
   </si>
@@ -34,6 +34,12 @@
   </si>
   <si>
     <t>Fairbanks</t>
+  </si>
+  <si>
+    <t>latitude</t>
+  </si>
+  <si>
+    <t>longitude</t>
   </si>
 </sst>
 </file>
@@ -372,37 +378,73 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:C6"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
-    </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C1" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B2">
+        <v>33.6594835</v>
+      </c>
+      <c r="C2">
+        <v>-117.9988026</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B3">
+        <v>33.6594835</v>
+      </c>
+      <c r="C3">
+        <v>-117.9988026</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B4">
+        <v>33.6594835</v>
+      </c>
+      <c r="C4">
+        <v>-117.9988026</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="B5">
+        <v>33.6594835</v>
+      </c>
+      <c r="C5">
+        <v>-117.9988026</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
+      </c>
+      <c r="B6">
+        <v>33.6594835</v>
+      </c>
+      <c r="C6">
+        <v>-117.9988026</v>
       </c>
     </row>
   </sheetData>

</xml_diff>